<commit_message>
EDW-33: pipeline v1 (parsers, OCR, table extraction, matching, multi-attachment merge), runner and scorer; recorded fixture/label corrections after run a1
Label correction: vat_mode mapping bug in the generator. Fixture correction: overlapping column headers in rendered pages. Baseline a0/a1 numbers kept in the report.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/benchmarks/attachment_intelligence/fixtures/files/f10.xlsx
+++ b/benchmarks/attachment_intelligence/fixtures/files/f10.xlsx
@@ -52,7 +52,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Количество</t>
+          <t xml:space="preserve">Кол-во</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -62,12 +62,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Цена за ед., руб.</t>
+          <t xml:space="preserve">Цена, руб.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Стоимость, руб.</t>
+          <t xml:space="preserve">Стоимость</t>
         </is>
       </c>
     </row>

</xml_diff>